<commit_message>
updated production tracking size-wise process fix
</commit_message>
<xml_diff>
--- a/Sonna_Order_Count.xlsx
+++ b/Sonna_Order_Count.xlsx
@@ -454,7 +454,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>210</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3">
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>420</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4">
@@ -487,10 +487,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>840</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5">
@@ -505,10 +505,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>630</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6">
@@ -523,16 +523,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>420</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ROSE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>420</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ROSE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>420</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ROSE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -577,16 +577,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>840</v>
+        <v>284</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ROSE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -595,16 +595,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>840</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ROSE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>420</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -634,13 +634,13 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>210</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -652,13 +652,13 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>210</v>
+        <v>284</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -667,16 +667,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>840</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -685,16 +685,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>630</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -706,7 +706,7 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>210</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -742,27 +742,27 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2520</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ROSE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2940</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2100</v>
+        <v>1420</v>
       </c>
     </row>
   </sheetData>

</xml_diff>